<commit_message>
Workflow Admin (Proses Input Kataloger Done)
</commit_message>
<xml_diff>
--- a/public/templates/template_materiil.xlsx
+++ b/public/templates/template_materiil.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Evan\Downloads\Kirim Evan\Kirim Evan\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Project Web\puskod-codification\public\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{39B59876-585E-4DA8-9916-6B82F94EA9E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D69D47B3-EFD0-428A-8AB8-5A4FC25A1151}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{6BED9FE3-C1D6-4B59-942D-6A7CDDE69BC4}"/>
   </bookViews>
@@ -79,7 +79,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
       <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
@@ -468,5 +467,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>